<commit_message>
feat: complete boutique website with authentic Naomika Design storefront, responsive cards, 3-photo galleries, and bespoke customization flow
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M34"/>
+  <dimension ref="A1:M32"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -442,31 +442,31 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>NDS-LW-102</v>
+        <v>NDS-LW-103</v>
       </c>
       <c r="B2" t="str">
-        <v>Red Satin Floral Embellished Ensemble</v>
+        <v>Regal Purple Zari Anarkali Gown</v>
       </c>
       <c r="C2" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D2" t="str">
-        <v>Festive Wear</v>
+        <v>Anarkalis</v>
       </c>
       <c r="E2">
-        <v>8500</v>
+        <v>17000</v>
       </c>
       <c r="F2">
-        <v>10500</v>
+        <v>21000</v>
       </c>
       <c r="G2" t="str">
-        <v>2.jpeg</v>
+        <v>3.jpeg</v>
       </c>
       <c r="H2" t="str">
-        <v>1.jpeg</v>
+        <v>4.jpeg</v>
       </c>
       <c r="I2" t="str">
-        <v>2.jpeg</v>
+        <v>3.jpeg</v>
       </c>
       <c r="J2" t="str">
         <v>In Stock</v>
@@ -475,7 +475,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L2" t="str">
-        <v>Luxurious red satin ensemble showcasing bold floral prints, flattering V-neckline, and intricate embellished detailing along borders with flowing sleeves.</v>
+        <v>Regal purple Anarkali gown featuring intricate floral embroidery, fitted embellished bodice, and sheer three-quarter sleeves for an elegant finish.</v>
       </c>
       <c r="M2" t="str">
         <v>Yes</v>
@@ -483,10 +483,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>NDS-LW-103</v>
+        <v>NDS-LW-104</v>
       </c>
       <c r="B3" t="str">
-        <v>Regal Purple Zari Anarkali Gown</v>
+        <v>Celestial Ivory &amp; Gold Anarkali</v>
       </c>
       <c r="C3" t="str">
         <v>Ladies Wear</v>
@@ -495,20 +495,20 @@
         <v>Anarkalis</v>
       </c>
       <c r="E3">
-        <v>17000</v>
+        <v>4900</v>
       </c>
       <c r="F3">
-        <v>21000</v>
+        <v>6200</v>
       </c>
       <c r="G3" t="str">
+        <v>4.jpeg</v>
+      </c>
+      <c r="H3" t="str">
         <v>3.jpeg</v>
       </c>
-      <c r="H3" t="str">
+      <c r="I3" t="str">
         <v>4.jpeg</v>
       </c>
-      <c r="I3" t="str">
-        <v>3.jpeg</v>
-      </c>
       <c r="J3" t="str">
         <v>In Stock</v>
       </c>
@@ -516,7 +516,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L3" t="str">
-        <v>Regal purple Anarkali gown featuring intricate floral embroidery, fitted embellished bodice, and sheer three-quarter sleeves for an elegant finish.</v>
+        <v>Elegant white Anarkali-inspired dress with delicate golden motifs, sheer full sleeves, and fine pleated drape for graceful festive movement.</v>
       </c>
       <c r="M3" t="str">
         <v>Yes</v>
@@ -524,31 +524,31 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>NDS-LW-104</v>
+        <v>NDS-LW-105</v>
       </c>
       <c r="B4" t="str">
-        <v>Celestial Ivory &amp; Gold Anarkali</v>
+        <v>Vibrant Red Organza Ensemble</v>
       </c>
       <c r="C4" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D4" t="str">
-        <v>Anarkalis</v>
+        <v>Festive Wear</v>
       </c>
       <c r="E4">
-        <v>4900</v>
+        <v>14200</v>
       </c>
       <c r="F4">
-        <v>6200</v>
+        <v>16500</v>
       </c>
       <c r="G4" t="str">
-        <v>4.jpeg</v>
+        <v>6.png</v>
       </c>
       <c r="H4" t="str">
-        <v>3.jpeg</v>
+        <v>5.png</v>
       </c>
       <c r="I4" t="str">
-        <v>4.jpeg</v>
+        <v>6.png</v>
       </c>
       <c r="J4" t="str">
         <v>In Stock</v>
@@ -557,7 +557,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L4" t="str">
-        <v>Elegant white Anarkali-inspired dress with delicate golden motifs, sheer full sleeves, and fine pleated drape for graceful festive movement.</v>
+        <v>Fitted crop top with vertical detailing, paired with a flowing skirt and sheer organza dupatta finished with silver-gold scalloped borders.</v>
       </c>
       <c r="M4" t="str">
         <v>Yes</v>
@@ -565,40 +565,40 @@
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>NDS-CU-301</v>
+        <v>NDS-LW-106</v>
       </c>
       <c r="B5" t="str">
-        <v>Ivory Corset Mermaid Haute Gown</v>
+        <v>Ivory Kerala Floral Kasavu Saree</v>
       </c>
       <c r="C5" t="str">
-        <v>Customization</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D5" t="str">
-        <v>Bespoke Couture</v>
+        <v>Sarees</v>
       </c>
       <c r="E5">
-        <v>24500</v>
+        <v>11500</v>
       </c>
       <c r="F5">
-        <v>30000</v>
+        <v>13900</v>
       </c>
       <c r="G5" t="str">
-        <v>5.png</v>
+        <v>7.png</v>
       </c>
       <c r="H5" t="str">
-        <v>6.png</v>
+        <v>8.png</v>
       </c>
       <c r="I5" t="str">
-        <v>5.png</v>
+        <v>7.png</v>
       </c>
       <c r="J5" t="str">
-        <v>Made to Order</v>
+        <v>In Stock</v>
       </c>
       <c r="K5" t="str">
-        <v>Haute Couture</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="L5" t="str">
-        <v>Sculpted corset bodice, sleek mermaid silhouette, refined gold vertical accent and subtle flared hem. A fusion of Kerala heritage and modern couture.</v>
+        <v>Graceful ivory handloom saree featuring soft botanical florals, complemented by authentic Kerala golden kasavu tissue zari borders.</v>
       </c>
       <c r="M5" t="str">
         <v>Yes</v>
@@ -606,31 +606,31 @@
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>NDS-LW-105</v>
+        <v>NDS-MW-201</v>
       </c>
       <c r="B6" t="str">
-        <v>Vibrant Red Organza Ensemble</v>
+        <v>Ivory Mundu &amp; Kurta Festive Set</v>
       </c>
       <c r="C6" t="str">
-        <v>Ladies Wear</v>
+        <v>Mens Wear</v>
       </c>
       <c r="D6" t="str">
-        <v>Festive Wear</v>
+        <v>Traditional Kasavu</v>
       </c>
       <c r="E6">
-        <v>14200</v>
+        <v>5800</v>
       </c>
       <c r="F6">
-        <v>16500</v>
+        <v>7000</v>
       </c>
       <c r="G6" t="str">
-        <v>6.png</v>
+        <v>8.png</v>
       </c>
       <c r="H6" t="str">
-        <v>5.png</v>
+        <v>7.png</v>
       </c>
       <c r="I6" t="str">
-        <v>6.png</v>
+        <v>8.png</v>
       </c>
       <c r="J6" t="str">
         <v>In Stock</v>
@@ -639,7 +639,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L6" t="str">
-        <v>Fitted crop top with vertical detailing, paired with a flowing skirt and sheer organza dupatta finished with silver-gold scalloped borders.</v>
+        <v>Traditional Kerala-inspired ensemble featuring a crisp ivory kurta with subtle golden vertical stripes, paired with matching kasavu mundu.</v>
       </c>
       <c r="M6" t="str">
         <v>Yes</v>
@@ -647,31 +647,31 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>NDS-LW-106</v>
+        <v>NDS-LW-107</v>
       </c>
       <c r="B7" t="str">
-        <v>Ivory Kerala Floral Kasavu Saree</v>
+        <v>Navy Brocade Halter Top &amp; Skirt</v>
       </c>
       <c r="C7" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D7" t="str">
-        <v>Sarees</v>
+        <v>Co-Ords</v>
       </c>
       <c r="E7">
-        <v>11500</v>
+        <v>9800</v>
       </c>
       <c r="F7">
-        <v>13900</v>
+        <v>12000</v>
       </c>
       <c r="G7" t="str">
-        <v>7.png</v>
+        <v>9.png</v>
       </c>
       <c r="H7" t="str">
-        <v>8.png</v>
+        <v>10.png</v>
       </c>
       <c r="I7" t="str">
-        <v>7.png</v>
+        <v>9.png</v>
       </c>
       <c r="J7" t="str">
         <v>In Stock</v>
@@ -680,7 +680,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L7" t="str">
-        <v>Graceful ivory handloom saree featuring soft botanical florals, complemented by authentic Kerala golden kasavu tissue zari borders.</v>
+        <v>Structured high halter neck crop top in navy blue brocade with gold floral weave, paired with a traditional ivory skirt.</v>
       </c>
       <c r="M7" t="str">
         <v>Yes</v>
@@ -688,40 +688,40 @@
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>NDS-MW-201</v>
+        <v>NDS-CU-302</v>
       </c>
       <c r="B8" t="str">
-        <v>Ivory Mundu &amp; Kurta Festive Set</v>
+        <v>Regal Maroon &amp; Champagne Bridal Lehenga</v>
       </c>
       <c r="C8" t="str">
-        <v>Mens Wear</v>
+        <v>Customization</v>
       </c>
       <c r="D8" t="str">
-        <v>Traditional Kasavu</v>
+        <v>Bespoke Couture</v>
       </c>
       <c r="E8">
-        <v>5800</v>
+        <v>48000</v>
       </c>
       <c r="F8">
-        <v>7000</v>
+        <v>58000</v>
       </c>
       <c r="G8" t="str">
-        <v>8.png</v>
+        <v>10.png</v>
       </c>
       <c r="H8" t="str">
-        <v>7.png</v>
+        <v>9.png</v>
       </c>
       <c r="I8" t="str">
-        <v>8.png</v>
+        <v>10.png</v>
       </c>
       <c r="J8" t="str">
-        <v>In Stock</v>
+        <v>Made to Order</v>
       </c>
       <c r="K8" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Haute Couture</v>
       </c>
       <c r="L8" t="str">
-        <v>Traditional Kerala-inspired ensemble featuring a crisp ivory kurta with subtle golden vertical stripes, paired with matching kasavu mundu.</v>
+        <v>Richly embellished maroon velvet blouse paired with luxurious champagne gold lehenga and ornate hand-stitched zardozi borders.</v>
       </c>
       <c r="M8" t="str">
         <v>Yes</v>
@@ -729,31 +729,31 @@
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>NDS-LW-107</v>
+        <v>NDS-LW-108</v>
       </c>
       <c r="B9" t="str">
-        <v>Navy Brocade Halter Top &amp; Skirt</v>
+        <v>Navy Blue V-Neck Flowing Anarkali</v>
       </c>
       <c r="C9" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D9" t="str">
-        <v>Co-Ords</v>
+        <v>Anarkalis</v>
       </c>
       <c r="E9">
-        <v>9800</v>
+        <v>12500</v>
       </c>
       <c r="F9">
-        <v>12000</v>
+        <v>15000</v>
       </c>
       <c r="G9" t="str">
-        <v>9.png</v>
+        <v>11.jpeg</v>
       </c>
       <c r="H9" t="str">
-        <v>10.png</v>
+        <v>12.jpeg</v>
       </c>
       <c r="I9" t="str">
-        <v>9.png</v>
+        <v>11.jpeg</v>
       </c>
       <c r="J9" t="str">
         <v>In Stock</v>
@@ -762,7 +762,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L9" t="str">
-        <v>Structured high halter neck crop top in navy blue brocade with gold floral weave, paired with a traditional ivory skirt.</v>
+        <v>Sleeveless V-neck bodice with subtle embroidered edging and fine vertical textured detailing. Flowing floor-length silhouette.</v>
       </c>
       <c r="M9" t="str">
         <v>Yes</v>
@@ -770,51 +770,51 @@
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>NDS-CU-302</v>
+        <v>NDS-LW-109</v>
       </c>
       <c r="B10" t="str">
-        <v>Regal Maroon &amp; Champagne Bridal Lehenga</v>
+        <v>Teal Wave Pattern Indo-Western Set</v>
       </c>
       <c r="C10" t="str">
-        <v>Customization</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D10" t="str">
-        <v>Bespoke Couture</v>
+        <v>Co-Ords</v>
       </c>
       <c r="E10">
-        <v>48000</v>
+        <v>9200</v>
       </c>
       <c r="F10">
-        <v>58000</v>
+        <v>11000</v>
       </c>
       <c r="G10" t="str">
-        <v>10.png</v>
+        <v>12.jpeg</v>
       </c>
       <c r="H10" t="str">
-        <v>9.png</v>
+        <v>11.jpeg</v>
       </c>
       <c r="I10" t="str">
-        <v>10.png</v>
+        <v>12.jpeg</v>
       </c>
       <c r="J10" t="str">
-        <v>Made to Order</v>
+        <v>In Stock</v>
       </c>
       <c r="K10" t="str">
-        <v>Haute Couture</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="L10" t="str">
-        <v>Richly embellished maroon velvet blouse paired with luxurious champagne gold lehenga and ornate hand-stitched zardozi borders.</v>
+        <v>Contemporary Indo-Western ensemble pairing a teal midi dress with an open-front overlay featuring an elegant blue-grey wave pattern.</v>
       </c>
       <c r="M10" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>NDS-LW-108</v>
+        <v>NDS-LW-110</v>
       </c>
       <c r="B11" t="str">
-        <v>Navy Blue V-Neck Flowing Anarkali</v>
+        <v>Royal Blue Pearl-Accented Anarkali</v>
       </c>
       <c r="C11" t="str">
         <v>Ladies Wear</v>
@@ -823,19 +823,19 @@
         <v>Anarkalis</v>
       </c>
       <c r="E11">
-        <v>12500</v>
+        <v>16800</v>
       </c>
       <c r="F11">
-        <v>15000</v>
+        <v>19500</v>
       </c>
       <c r="G11" t="str">
-        <v>11.jpeg</v>
+        <v>13.jpeg</v>
       </c>
       <c r="H11" t="str">
-        <v>12.jpeg</v>
+        <v>14.jpeg</v>
       </c>
       <c r="I11" t="str">
-        <v>11.jpeg</v>
+        <v>13.jpeg</v>
       </c>
       <c r="J11" t="str">
         <v>In Stock</v>
@@ -844,7 +844,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L11" t="str">
-        <v>Sleeveless V-neck bodice with subtle embroidered edging and fine vertical textured detailing. Flowing floor-length silhouette.</v>
+        <v>Fitted kurta with square neckline, delicate pearl-like embellishment, scalloped hem, sheer sleeves, and a matching voluminous dupatta.</v>
       </c>
       <c r="M11" t="str">
         <v>Yes</v>
@@ -852,31 +852,31 @@
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>NDS-LW-109</v>
+        <v>NDS-LW-111</v>
       </c>
       <c r="B12" t="str">
-        <v>Teal Wave Pattern Indo-Western Set</v>
+        <v>Teal Floor-Length Flare Anarkali</v>
       </c>
       <c r="C12" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D12" t="str">
-        <v>Co-Ords</v>
+        <v>Anarkalis</v>
       </c>
       <c r="E12">
-        <v>9200</v>
+        <v>13900</v>
       </c>
       <c r="F12">
-        <v>11000</v>
+        <v>16000</v>
       </c>
       <c r="G12" t="str">
-        <v>12.jpeg</v>
+        <v>14.jpeg</v>
       </c>
       <c r="H12" t="str">
-        <v>11.jpeg</v>
+        <v>13.jpeg</v>
       </c>
       <c r="I12" t="str">
-        <v>12.jpeg</v>
+        <v>14.jpeg</v>
       </c>
       <c r="J12" t="str">
         <v>In Stock</v>
@@ -885,7 +885,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L12" t="str">
-        <v>Contemporary Indo-Western ensemble pairing a teal midi dress with an open-front overlay featuring an elegant blue-grey wave pattern.</v>
+        <v>Fitted bodice, front tie detailing, and voluminous floor-length flare. Sheer matching dupatta finished with silver-toned edging.</v>
       </c>
       <c r="M12" t="str">
         <v>No</v>
@@ -893,31 +893,31 @@
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>NDS-LW-110</v>
+        <v>NDS-LW-112</v>
       </c>
       <c r="B13" t="str">
-        <v>Royal Blue Pearl-Accented Anarkali</v>
+        <v>Teal &amp; Maroon Peplum Palazzo Set</v>
       </c>
       <c r="C13" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D13" t="str">
-        <v>Anarkalis</v>
+        <v>Festive Wear</v>
       </c>
       <c r="E13">
-        <v>16800</v>
+        <v>11000</v>
       </c>
       <c r="F13">
-        <v>19500</v>
+        <v>13500</v>
       </c>
       <c r="G13" t="str">
-        <v>13.jpeg</v>
+        <v>15.jpeg</v>
       </c>
       <c r="H13" t="str">
-        <v>14.jpeg</v>
+        <v>16.jpeg</v>
       </c>
       <c r="I13" t="str">
-        <v>13.jpeg</v>
+        <v>15.jpeg</v>
       </c>
       <c r="J13" t="str">
         <v>In Stock</v>
@@ -926,7 +926,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L13" t="str">
-        <v>Fitted kurta with square neckline, delicate pearl-like embellishment, scalloped hem, sheer sleeves, and a matching voluminous dupatta.</v>
+        <v>Structured teal peplum-style kurti with delicate gold motifs, maroon border, and a voluminous ivory palazzo skirt.</v>
       </c>
       <c r="M13" t="str">
         <v>Yes</v>
@@ -934,31 +934,31 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>NDS-LW-111</v>
+        <v>NDS-LW-113</v>
       </c>
       <c r="B14" t="str">
-        <v>Teal Floor-Length Flare Anarkali</v>
+        <v>Emerald &amp; Gold Ivory Flared Set</v>
       </c>
       <c r="C14" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D14" t="str">
-        <v>Anarkalis</v>
+        <v>Festive Wear</v>
       </c>
       <c r="E14">
-        <v>13900</v>
+        <v>14500</v>
       </c>
       <c r="F14">
-        <v>16000</v>
+        <v>17000</v>
       </c>
       <c r="G14" t="str">
-        <v>14.jpeg</v>
+        <v>16.jpeg</v>
       </c>
       <c r="H14" t="str">
-        <v>13.jpeg</v>
+        <v>15.jpeg</v>
       </c>
       <c r="I14" t="str">
-        <v>14.jpeg</v>
+        <v>16.jpeg</v>
       </c>
       <c r="J14" t="str">
         <v>In Stock</v>
@@ -967,39 +967,39 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L14" t="str">
-        <v>Fitted bodice, front tie detailing, and voluminous floor-length flare. Sheer matching dupatta finished with silver-toned edging.</v>
+        <v>Rich emerald-green blouse with delicate gold motifs, flowing ivory flared skirt, and sheer green dupatta with ornate gold border.</v>
       </c>
       <c r="M14" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>NDS-LW-112</v>
+        <v>NDS-LW-114</v>
       </c>
       <c r="B15" t="str">
-        <v>Teal &amp; Maroon Peplum Palazzo Set</v>
+        <v>Charming Pink Tulle Party Gown</v>
       </c>
       <c r="C15" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D15" t="str">
-        <v>Festive Wear</v>
+        <v>Gowns</v>
       </c>
       <c r="E15">
-        <v>11000</v>
+        <v>15500</v>
       </c>
       <c r="F15">
-        <v>13500</v>
+        <v>18000</v>
       </c>
       <c r="G15" t="str">
-        <v>15.jpeg</v>
+        <v>17.jpeg</v>
       </c>
       <c r="H15" t="str">
-        <v>16.jpeg</v>
+        <v>18.jpeg</v>
       </c>
       <c r="I15" t="str">
-        <v>15.jpeg</v>
+        <v>17.jpeg</v>
       </c>
       <c r="J15" t="str">
         <v>In Stock</v>
@@ -1008,39 +1008,39 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L15" t="str">
-        <v>Structured teal peplum-style kurti with delicate gold motifs, maroon border, and a voluminous ivory palazzo skirt.</v>
+        <v>Embellished bodice with floral and sequin detailing, voluminous layered tulle skirt, and whimsical sheer cape-style sleeves.</v>
       </c>
       <c r="M15" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>NDS-LW-113</v>
+        <v>NDS-LW-115</v>
       </c>
       <c r="B16" t="str">
-        <v>Emerald &amp; Gold Ivory Flared Set</v>
+        <v>Navy Blue Checked Lehenga Set</v>
       </c>
       <c r="C16" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D16" t="str">
-        <v>Festive Wear</v>
+        <v>Lehengas</v>
       </c>
       <c r="E16">
-        <v>14500</v>
+        <v>28000</v>
       </c>
       <c r="F16">
-        <v>17000</v>
+        <v>34000</v>
       </c>
       <c r="G16" t="str">
-        <v>16.jpeg</v>
+        <v>18.jpeg</v>
       </c>
       <c r="H16" t="str">
-        <v>15.jpeg</v>
+        <v>17.jpeg</v>
       </c>
       <c r="I16" t="str">
-        <v>16.jpeg</v>
+        <v>18.jpeg</v>
       </c>
       <c r="J16" t="str">
         <v>In Stock</v>
@@ -1049,7 +1049,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L16" t="str">
-        <v>Rich emerald-green blouse with delicate gold motifs, flowing ivory flared skirt, and sheer green dupatta with ornate gold border.</v>
+        <v>Structured square-neck crop blouse and voluminous flared skirt with subtle checked texture and ornate antique-gold border.</v>
       </c>
       <c r="M16" t="str">
         <v>Yes</v>
@@ -1057,31 +1057,31 @@
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>NDS-LW-114</v>
+        <v>NDS-LW-116</v>
       </c>
       <c r="B17" t="str">
-        <v>Charming Pink Tulle Party Gown</v>
+        <v>Pastel Pink Tiered Midi Dress</v>
       </c>
       <c r="C17" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D17" t="str">
-        <v>Gowns</v>
+        <v>Festive Wear</v>
       </c>
       <c r="E17">
-        <v>15500</v>
+        <v>7500</v>
       </c>
       <c r="F17">
-        <v>18000</v>
+        <v>9000</v>
       </c>
       <c r="G17" t="str">
-        <v>17.jpeg</v>
+        <v>19.jpeg</v>
       </c>
       <c r="H17" t="str">
-        <v>18.jpeg</v>
+        <v>20.jpeg</v>
       </c>
       <c r="I17" t="str">
-        <v>17.jpeg</v>
+        <v>19.jpeg</v>
       </c>
       <c r="J17" t="str">
         <v>In Stock</v>
@@ -1090,7 +1090,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L17" t="str">
-        <v>Embellished bodice with floral and sequin detailing, voluminous layered tulle skirt, and whimsical sheer cape-style sleeves.</v>
+        <v>Square neckline, softly gathered sleeves, and flowing tiered silhouette with delicate floral embroidery along panels.</v>
       </c>
       <c r="M17" t="str">
         <v>No</v>
@@ -1098,31 +1098,31 @@
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>NDS-LW-115</v>
+        <v>NDS-LW-117</v>
       </c>
       <c r="B18" t="str">
-        <v>Navy Blue Checked Lehenga Set</v>
+        <v>Olive &amp; Magenta Tiered Fusion Dress</v>
       </c>
       <c r="C18" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D18" t="str">
-        <v>Lehengas</v>
+        <v>Festive Wear</v>
       </c>
       <c r="E18">
-        <v>28000</v>
+        <v>8800</v>
       </c>
       <c r="F18">
-        <v>34000</v>
+        <v>10500</v>
       </c>
       <c r="G18" t="str">
-        <v>18.jpeg</v>
+        <v>20.jpeg</v>
       </c>
       <c r="H18" t="str">
-        <v>17.jpeg</v>
+        <v>19.jpeg</v>
       </c>
       <c r="I18" t="str">
-        <v>18.jpeg</v>
+        <v>20.jpeg</v>
       </c>
       <c r="J18" t="str">
         <v>In Stock</v>
@@ -1131,39 +1131,39 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L18" t="str">
-        <v>Structured square-neck crop blouse and voluminous flared skirt with subtle checked texture and ornate antique-gold border.</v>
+        <v>Contrasting olive-green and deep magenta panels in a pleated silhouette with delicate gold waistband and ornate hem border.</v>
       </c>
       <c r="M18" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>NDS-LW-116</v>
+        <v>NDS-LW-118</v>
       </c>
       <c r="B19" t="str">
-        <v>Pastel Pink Tiered Midi Dress</v>
+        <v>Coral Pink Pleated Anarkali</v>
       </c>
       <c r="C19" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D19" t="str">
-        <v>Festive Wear</v>
+        <v>Anarkalis</v>
       </c>
       <c r="E19">
-        <v>7500</v>
+        <v>13200</v>
       </c>
       <c r="F19">
-        <v>9000</v>
+        <v>15800</v>
       </c>
       <c r="G19" t="str">
-        <v>19.jpeg</v>
+        <v>21.jpeg</v>
       </c>
       <c r="H19" t="str">
-        <v>20.jpeg</v>
+        <v>22.jpeg</v>
       </c>
       <c r="I19" t="str">
-        <v>19.jpeg</v>
+        <v>21.jpeg</v>
       </c>
       <c r="J19" t="str">
         <v>In Stock</v>
@@ -1172,18 +1172,18 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L19" t="str">
-        <v>Square neckline, softly gathered sleeves, and flowing tiered silhouette with delicate floral embroidery along panels.</v>
+        <v>Delicately embroidered bodice with keyhole neckline, finely pleated floor-length skirt, and sheer pearl-edged dupatta.</v>
       </c>
       <c r="M19" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>NDS-LW-117</v>
+        <v>NDS-LW-119</v>
       </c>
       <c r="B20" t="str">
-        <v>Olive &amp; Magenta Tiered Fusion Dress</v>
+        <v>Vibrant Red Puff-Sleeve Maxi Dress</v>
       </c>
       <c r="C20" t="str">
         <v>Ladies Wear</v>
@@ -1192,19 +1192,19 @@
         <v>Festive Wear</v>
       </c>
       <c r="E20">
-        <v>8800</v>
+        <v>12800</v>
       </c>
       <c r="F20">
-        <v>10500</v>
+        <v>15000</v>
       </c>
       <c r="G20" t="str">
-        <v>20.jpeg</v>
+        <v>22.jpeg</v>
       </c>
       <c r="H20" t="str">
-        <v>19.jpeg</v>
+        <v>21.jpeg</v>
       </c>
       <c r="I20" t="str">
-        <v>20.jpeg</v>
+        <v>22.jpeg</v>
       </c>
       <c r="J20" t="str">
         <v>In Stock</v>
@@ -1213,7 +1213,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L20" t="str">
-        <v>Contrasting olive-green and deep magenta panels in a pleated silhouette with delicate gold waistband and ornate hem border.</v>
+        <v>All-over texture, flattering V-neckline, dramatic puff sleeves with ruffled trims, and metallic woven waistband.</v>
       </c>
       <c r="M20" t="str">
         <v>No</v>
@@ -1221,31 +1221,31 @@
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>NDS-LW-118</v>
+        <v>NDS-LW-120</v>
       </c>
       <c r="B21" t="str">
-        <v>Coral Pink Pleated Anarkali</v>
+        <v>Monochrome Black &amp; Rose Evening Dress</v>
       </c>
       <c r="C21" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D21" t="str">
-        <v>Anarkalis</v>
+        <v>Gowns</v>
       </c>
       <c r="E21">
-        <v>13200</v>
+        <v>16500</v>
       </c>
       <c r="F21">
-        <v>15800</v>
+        <v>19500</v>
       </c>
       <c r="G21" t="str">
-        <v>21.jpeg</v>
+        <v>23.jpeg</v>
       </c>
       <c r="H21" t="str">
-        <v>22.jpeg</v>
+        <v>24.jpeg</v>
       </c>
       <c r="I21" t="str">
-        <v>21.jpeg</v>
+        <v>23.jpeg</v>
       </c>
       <c r="J21" t="str">
         <v>In Stock</v>
@@ -1254,7 +1254,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L21" t="str">
-        <v>Delicately embroidered bodice with keyhole neckline, finely pleated floor-length skirt, and sheer pearl-edged dupatta.</v>
+        <v>Fitted bodice with graceful off-shoulder neckline, statement white draped collar, and oversized fabric rose.</v>
       </c>
       <c r="M21" t="str">
         <v>Yes</v>
@@ -1262,31 +1262,31 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>NDS-LW-119</v>
+        <v>NDS-LW-121</v>
       </c>
       <c r="B22" t="str">
-        <v>Vibrant Red Puff-Sleeve Maxi Dress</v>
+        <v>Lavender Ombré Pleated Statement Dress</v>
       </c>
       <c r="C22" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D22" t="str">
-        <v>Festive Wear</v>
+        <v>Gowns</v>
       </c>
       <c r="E22">
-        <v>12800</v>
+        <v>14800</v>
       </c>
       <c r="F22">
-        <v>15000</v>
+        <v>17500</v>
       </c>
       <c r="G22" t="str">
-        <v>22.jpeg</v>
+        <v>24.jpeg</v>
       </c>
       <c r="H22" t="str">
-        <v>21.jpeg</v>
+        <v>23.jpeg</v>
       </c>
       <c r="I22" t="str">
-        <v>22.jpeg</v>
+        <v>24.jpeg</v>
       </c>
       <c r="J22" t="str">
         <v>In Stock</v>
@@ -1295,7 +1295,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L22" t="str">
-        <v>All-over texture, flattering V-neckline, dramatic puff sleeves with ruffled trims, and metallic woven waistband.</v>
+        <v>High pleated neckline, lavender-to-aqua ombré transition, and luminous fluid pleats creating graceful movement.</v>
       </c>
       <c r="M22" t="str">
         <v>No</v>
@@ -1303,40 +1303,40 @@
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>NDS-LW-120</v>
+        <v>NDS-CU-303</v>
       </c>
       <c r="B23" t="str">
-        <v>Monochrome Black &amp; Rose Evening Dress</v>
+        <v>Nature-Inspired Capsule Haute Ensemble</v>
       </c>
       <c r="C23" t="str">
-        <v>Ladies Wear</v>
+        <v>Customization</v>
       </c>
       <c r="D23" t="str">
-        <v>Gowns</v>
+        <v>Bespoke Couture</v>
       </c>
       <c r="E23">
-        <v>16500</v>
+        <v>38000</v>
       </c>
       <c r="F23">
-        <v>19500</v>
+        <v>45000</v>
       </c>
       <c r="G23" t="str">
-        <v>23.jpeg</v>
+        <v>25.jpeg</v>
       </c>
       <c r="H23" t="str">
-        <v>24.jpeg</v>
+        <v>26.jpeg</v>
       </c>
       <c r="I23" t="str">
-        <v>23.jpeg</v>
+        <v>25.jpeg</v>
       </c>
       <c r="J23" t="str">
-        <v>In Stock</v>
+        <v>Made to Order</v>
       </c>
       <c r="K23" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Haute Couture</v>
       </c>
       <c r="L23" t="str">
-        <v>Fitted bodice with graceful off-shoulder neckline, statement white draped collar, and oversized fabric rose.</v>
+        <v>Four coordinated silhouettes in ivory, powder blue, and teal with delicate metallic detailing and feminine movement.</v>
       </c>
       <c r="M23" t="str">
         <v>Yes</v>
@@ -1344,31 +1344,31 @@
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>NDS-LW-121</v>
+        <v>NDS-MW-202</v>
       </c>
       <c r="B24" t="str">
-        <v>Lavender Ombré Pleated Statement Dress</v>
+        <v>Black &amp; Silver Motif Royal Kurta Set</v>
       </c>
       <c r="C24" t="str">
-        <v>Ladies Wear</v>
+        <v>Mens Wear</v>
       </c>
       <c r="D24" t="str">
-        <v>Gowns</v>
+        <v>Kurtas</v>
       </c>
       <c r="E24">
-        <v>14800</v>
+        <v>7800</v>
       </c>
       <c r="F24">
-        <v>17500</v>
+        <v>9500</v>
       </c>
       <c r="G24" t="str">
-        <v>24.jpeg</v>
+        <v>26.jpeg</v>
       </c>
       <c r="H24" t="str">
-        <v>23.jpeg</v>
+        <v>8.png</v>
       </c>
       <c r="I24" t="str">
-        <v>24.jpeg</v>
+        <v>26.jpeg</v>
       </c>
       <c r="J24" t="str">
         <v>In Stock</v>
@@ -1377,48 +1377,48 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L24" t="str">
-        <v>High pleated neckline, lavender-to-aqua ombré transition, and luminous fluid pleats creating graceful movement.</v>
+        <v>Subtle silver-toned vertical motifs, structured mandarin collar, statement buttons, and intricately patterned borders.</v>
       </c>
       <c r="M24" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>NDS-CU-303</v>
+        <v>NDS-MW-203</v>
       </c>
       <c r="B25" t="str">
-        <v>Nature-Inspired Capsule Haute Ensemble</v>
+        <v>Royal Kerala Kasavu Groom Mundu Set</v>
       </c>
       <c r="C25" t="str">
-        <v>Customization</v>
+        <v>Mens Wear</v>
       </c>
       <c r="D25" t="str">
-        <v>Bespoke Couture</v>
+        <v>Traditional Kasavu</v>
       </c>
       <c r="E25">
-        <v>38000</v>
+        <v>6200</v>
       </c>
       <c r="F25">
-        <v>45000</v>
+        <v>7500</v>
       </c>
       <c r="G25" t="str">
-        <v>25.jpeg</v>
+        <v>8.png</v>
       </c>
       <c r="H25" t="str">
-        <v>26.jpeg</v>
+        <v>7.png</v>
       </c>
       <c r="I25" t="str">
-        <v>25.jpeg</v>
+        <v>8.png</v>
       </c>
       <c r="J25" t="str">
-        <v>Made to Order</v>
+        <v>In Stock</v>
       </c>
       <c r="K25" t="str">
-        <v>Haute Couture</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="L25" t="str">
-        <v>Four coordinated silhouettes in ivory, powder blue, and teal with delicate metallic detailing and feminine movement.</v>
+        <v>Handwoven Balaramapuram fine cotton double mundu with pure gold kasavu border and matching ceremonial angavastram.</v>
       </c>
       <c r="M25" t="str">
         <v>Yes</v>
@@ -1426,31 +1426,31 @@
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>NDS-MW-202</v>
+        <v>NDS-MW-204</v>
       </c>
       <c r="B26" t="str">
-        <v>Black &amp; Silver Motif Royal Kurta Set</v>
+        <v>Obsidian Black Velvet Bandhgala Suit</v>
       </c>
       <c r="C26" t="str">
         <v>Mens Wear</v>
       </c>
       <c r="D26" t="str">
-        <v>Kurtas</v>
+        <v>Suits &amp; Blazers</v>
       </c>
       <c r="E26">
-        <v>7800</v>
+        <v>24500</v>
       </c>
       <c r="F26">
-        <v>9500</v>
+        <v>29000</v>
       </c>
       <c r="G26" t="str">
+        <v>10.png</v>
+      </c>
+      <c r="H26" t="str">
         <v>26.jpeg</v>
       </c>
-      <c r="H26" t="str">
-        <v>8.png</v>
-      </c>
       <c r="I26" t="str">
-        <v>26.jpeg</v>
+        <v>10.png</v>
       </c>
       <c r="J26" t="str">
         <v>In Stock</v>
@@ -1459,7 +1459,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L26" t="str">
-        <v>Subtle silver-toned vertical motifs, structured mandarin collar, statement buttons, and intricately patterned borders.</v>
+        <v>Structured Jodhpuri Bandhgala in micro-velvet with antique gold crest buttons and tapered formal trousers.</v>
       </c>
       <c r="M26" t="str">
         <v>Yes</v>
@@ -1467,31 +1467,31 @@
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>NDS-MW-203</v>
+        <v>NDS-MW-205</v>
       </c>
       <c r="B27" t="str">
-        <v>Royal Kerala Kasavu Groom Mundu Set</v>
+        <v>Champagne Raw Silk Festive Kurta</v>
       </c>
       <c r="C27" t="str">
         <v>Mens Wear</v>
       </c>
       <c r="D27" t="str">
-        <v>Traditional Kasavu</v>
+        <v>Kurtas</v>
       </c>
       <c r="E27">
-        <v>6200</v>
+        <v>6900</v>
       </c>
       <c r="F27">
-        <v>7500</v>
+        <v>8200</v>
       </c>
       <c r="G27" t="str">
+        <v>26.jpeg</v>
+      </c>
+      <c r="H27" t="str">
         <v>8.png</v>
       </c>
-      <c r="H27" t="str">
-        <v>7.png</v>
-      </c>
       <c r="I27" t="str">
-        <v>8.png</v>
+        <v>9.png</v>
       </c>
       <c r="J27" t="str">
         <v>In Stock</v>
@@ -1500,39 +1500,39 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L27" t="str">
-        <v>Handwoven Balaramapuram fine cotton double mundu with pure gold kasavu border and matching ceremonial angavastram.</v>
+        <v>Shimmering champagne raw silk knee-length kurta with concealed placket and hand-embroidered collar detailing.</v>
       </c>
       <c r="M27" t="str">
-        <v>Yes</v>
+        <v>No</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>NDS-MW-204</v>
+        <v>NDS-MW-206</v>
       </c>
       <c r="B28" t="str">
-        <v>Obsidian Black Velvet Bandhgala Suit</v>
+        <v>Midnight Navy Brocade Nehru Jacket</v>
       </c>
       <c r="C28" t="str">
         <v>Mens Wear</v>
       </c>
       <c r="D28" t="str">
-        <v>Suits &amp; Blazers</v>
+        <v>Kurtas</v>
       </c>
       <c r="E28">
-        <v>24500</v>
+        <v>8500</v>
       </c>
       <c r="F28">
-        <v>29000</v>
+        <v>10200</v>
       </c>
       <c r="G28" t="str">
-        <v>10.png</v>
+        <v>9.png</v>
       </c>
       <c r="H28" t="str">
-        <v>26.jpeg</v>
+        <v>8.png</v>
       </c>
       <c r="I28" t="str">
-        <v>10.png</v>
+        <v>9.png</v>
       </c>
       <c r="J28" t="str">
         <v>In Stock</v>
@@ -1541,7 +1541,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L28" t="str">
-        <v>Structured Jodhpuri Bandhgala in micro-velvet with antique gold crest buttons and tapered formal trousers.</v>
+        <v>Sleeveless Nehru bundi jacket in navy floral brocade weave layered over a crisp ivory linen kurta.</v>
       </c>
       <c r="M28" t="str">
         <v>Yes</v>
@@ -1549,31 +1549,31 @@
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>NDS-MW-205</v>
+        <v>NDS-MW-207</v>
       </c>
       <c r="B29" t="str">
-        <v>Champagne Raw Silk Festive Kurta</v>
+        <v>Pure White French Linen Tailored Shirt</v>
       </c>
       <c r="C29" t="str">
         <v>Mens Wear</v>
       </c>
       <c r="D29" t="str">
-        <v>Kurtas</v>
+        <v>Shirts</v>
       </c>
       <c r="E29">
-        <v>6900</v>
+        <v>3800</v>
       </c>
       <c r="F29">
-        <v>8200</v>
+        <v>4600</v>
       </c>
       <c r="G29" t="str">
-        <v>26.jpeg</v>
+        <v>8.png</v>
       </c>
       <c r="H29" t="str">
-        <v>8.png</v>
+        <v>9.png</v>
       </c>
       <c r="I29" t="str">
-        <v>9.png</v>
+        <v>10.png</v>
       </c>
       <c r="J29" t="str">
         <v>In Stock</v>
@@ -1582,7 +1582,7 @@
         <v>Fresh Arrivals</v>
       </c>
       <c r="L29" t="str">
-        <v>Shimmering champagne raw silk knee-length kurta with concealed placket and hand-embroidered collar detailing.</v>
+        <v>Breathable pure linen tailored shirt with mother-of-pearl buttons and mandarin collar, made for Kerala weather.</v>
       </c>
       <c r="M29" t="str">
         <v>No</v>
@@ -1590,40 +1590,40 @@
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>NDS-MW-206</v>
+        <v>NDS-CU-304</v>
       </c>
       <c r="B30" t="str">
-        <v>Midnight Navy Brocade Nehru Jacket</v>
+        <v>Bespoke Royal Heritage Zardozi Sherwani</v>
       </c>
       <c r="C30" t="str">
-        <v>Mens Wear</v>
+        <v>Customization</v>
       </c>
       <c r="D30" t="str">
-        <v>Kurtas</v>
+        <v>Bespoke Couture</v>
       </c>
       <c r="E30">
-        <v>8500</v>
+        <v>52000</v>
       </c>
       <c r="F30">
-        <v>10200</v>
+        <v>62000</v>
       </c>
       <c r="G30" t="str">
-        <v>9.png</v>
+        <v>8.png</v>
       </c>
       <c r="H30" t="str">
+        <v>10.png</v>
+      </c>
+      <c r="I30" t="str">
         <v>8.png</v>
       </c>
-      <c r="I30" t="str">
-        <v>9.png</v>
-      </c>
       <c r="J30" t="str">
-        <v>In Stock</v>
+        <v>Made to Order</v>
       </c>
       <c r="K30" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Haute Couture</v>
       </c>
       <c r="L30" t="str">
-        <v>Sleeveless Nehru bundi jacket in navy floral brocade weave layered over a crisp ivory linen kurta.</v>
+        <v>Handcrafted on pure Matka silk with customized monogramming and royal bullion gold embroidery.</v>
       </c>
       <c r="M30" t="str">
         <v>Yes</v>
@@ -1631,51 +1631,51 @@
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>NDS-MW-207</v>
+        <v>NDS-CU-305</v>
       </c>
       <c r="B31" t="str">
-        <v>Pure White French Linen Tailored Shirt</v>
+        <v>Bespoke Kerala Kasavu Corset Bridal Saree</v>
       </c>
       <c r="C31" t="str">
-        <v>Mens Wear</v>
+        <v>Customization</v>
       </c>
       <c r="D31" t="str">
-        <v>Shirts</v>
+        <v>Bespoke Couture</v>
       </c>
       <c r="E31">
-        <v>3800</v>
+        <v>42000</v>
       </c>
       <c r="F31">
-        <v>4600</v>
+        <v>50000</v>
       </c>
       <c r="G31" t="str">
-        <v>8.png</v>
+        <v>7.png</v>
       </c>
       <c r="H31" t="str">
-        <v>9.png</v>
+        <v>5.png</v>
       </c>
       <c r="I31" t="str">
-        <v>10.png</v>
+        <v>7.png</v>
       </c>
       <c r="J31" t="str">
-        <v>In Stock</v>
+        <v>Made to Order</v>
       </c>
       <c r="K31" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Made to Measure</v>
       </c>
       <c r="L31" t="str">
-        <v>Breathable pure linen tailored shirt with mother-of-pearl buttons and mandarin collar, made for Kerala weather.</v>
+        <v>Traditional Balaramapuram pure gold kasavu reimagined as a contemporary bridal corseted drape.</v>
       </c>
       <c r="M31" t="str">
-        <v>No</v>
+        <v>Yes</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>NDS-CU-304</v>
+        <v>NDS-CU-306</v>
       </c>
       <c r="B32" t="str">
-        <v>Bespoke Royal Heritage Zardozi Sherwani</v>
+        <v>The Sovereign Gold 3D Atelier Creation</v>
       </c>
       <c r="C32" t="str">
         <v>Customization</v>
@@ -1684,118 +1684,36 @@
         <v>Bespoke Couture</v>
       </c>
       <c r="E32">
-        <v>52000</v>
+        <v>62000</v>
       </c>
       <c r="F32">
-        <v>62000</v>
+        <v>72000</v>
       </c>
       <c r="G32" t="str">
-        <v>8.png</v>
+        <v>5.png</v>
       </c>
       <c r="H32" t="str">
-        <v>10.png</v>
+        <v>1.jpeg</v>
       </c>
       <c r="I32" t="str">
-        <v>8.png</v>
+        <v>5.png</v>
       </c>
       <c r="J32" t="str">
         <v>Made to Order</v>
       </c>
       <c r="K32" t="str">
-        <v>Haute Couture</v>
+        <v>3D Atelier Piece</v>
       </c>
       <c r="L32" t="str">
-        <v>Handcrafted on pure Matka silk with customized monogramming and royal bullion gold embroidery.</v>
+        <v>Masterpiece sculpted silhouette rendered in real-time 3D, individually tailored to client measurements.</v>
       </c>
       <c r="M32" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="str">
-        <v>NDS-CU-305</v>
-      </c>
-      <c r="B33" t="str">
-        <v>Bespoke Kerala Kasavu Corset Bridal Saree</v>
-      </c>
-      <c r="C33" t="str">
-        <v>Customization</v>
-      </c>
-      <c r="D33" t="str">
-        <v>Bespoke Couture</v>
-      </c>
-      <c r="E33">
-        <v>42000</v>
-      </c>
-      <c r="F33">
-        <v>50000</v>
-      </c>
-      <c r="G33" t="str">
-        <v>7.png</v>
-      </c>
-      <c r="H33" t="str">
-        <v>5.png</v>
-      </c>
-      <c r="I33" t="str">
-        <v>7.png</v>
-      </c>
-      <c r="J33" t="str">
-        <v>Made to Order</v>
-      </c>
-      <c r="K33" t="str">
-        <v>Made to Measure</v>
-      </c>
-      <c r="L33" t="str">
-        <v>Traditional Balaramapuram pure gold kasavu reimagined as a contemporary bridal corseted drape.</v>
-      </c>
-      <c r="M33" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="str">
-        <v>NDS-CU-306</v>
-      </c>
-      <c r="B34" t="str">
-        <v>The Sovereign Gold 3D Atelier Creation</v>
-      </c>
-      <c r="C34" t="str">
-        <v>Customization</v>
-      </c>
-      <c r="D34" t="str">
-        <v>Bespoke Couture</v>
-      </c>
-      <c r="E34">
-        <v>62000</v>
-      </c>
-      <c r="F34">
-        <v>72000</v>
-      </c>
-      <c r="G34" t="str">
-        <v>5.png</v>
-      </c>
-      <c r="H34" t="str">
-        <v>1.jpeg</v>
-      </c>
-      <c r="I34" t="str">
-        <v>5.png</v>
-      </c>
-      <c r="J34" t="str">
-        <v>Made to Order</v>
-      </c>
-      <c r="K34" t="str">
-        <v>3D Atelier Piece</v>
-      </c>
-      <c r="L34" t="str">
-        <v>Masterpiece sculpted silhouette rendered in real-time 3D, individually tailored to client measurements.</v>
-      </c>
-      <c r="M34" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M34"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M32"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Curated Gallery section with category filter tabs (Gallery, Ladies, Mens, Jewellery, Customization), Newest First sorting, and click-to-card quick view
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M6"/>
+  <dimension ref="A1:M8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -648,9 +648,91 @@
         <v>Yes</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>NDS-JW-1001</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Royal Antique Temple Jewellery Choker Set</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D7" t="str">
+        <v>Bridal Chokers</v>
+      </c>
+      <c r="E7">
+        <v>18500</v>
+      </c>
+      <c r="F7">
+        <v>22000</v>
+      </c>
+      <c r="G7" t="str">
+        <v>kerala_bridal_jewellery.jpg</v>
+      </c>
+      <c r="H7" t="str">
+        <v>kerala_bridal_jewellery.jpg</v>
+      </c>
+      <c r="I7" t="str">
+        <v>kerala_bridal_jewellery.jpg</v>
+      </c>
+      <c r="J7" t="str">
+        <v>In Stock</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Curated Release</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Authentic 22K antique gold finish temple jewellery bridal choker necklace adorned with radiant ruby-red stones, emerald accents, south sea pearls, and matching handcrafted jhumkas.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>NDS-JW-1002</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Heritage Kasavu Coin Necklace &amp; Royal Bangles</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Jewellery</v>
+      </c>
+      <c r="D8" t="str">
+        <v>Temple Jewellery</v>
+      </c>
+      <c r="E8">
+        <v>14200</v>
+      </c>
+      <c r="F8">
+        <v>16500</v>
+      </c>
+      <c r="G8" t="str">
+        <v>kerala_bridal_bangles.jpg</v>
+      </c>
+      <c r="H8" t="str">
+        <v>kerala_bridal_bangles.jpg</v>
+      </c>
+      <c r="I8" t="str">
+        <v>kerala_bridal_bangles.jpg</v>
+      </c>
+      <c r="J8" t="str">
+        <v>In Stock</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Curated Release</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Traditional Kerala Palakka and Kasavu coin necklace paired with intricately sculpted antique temple kadas featuring Goddess Lakshmi motifs and gemstone inlays.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Remove jewellery sections, remove subcategories, and unify product codes starting from P201 sequentially
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:L6"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,39 +410,36 @@
         <v>Category</v>
       </c>
       <c r="D1" t="str">
-        <v>Subcategory</v>
+        <v>Price</v>
       </c>
       <c r="E1" t="str">
-        <v>Price</v>
+        <v>Original Price</v>
       </c>
       <c r="F1" t="str">
-        <v>Original Price</v>
+        <v>Image 1</v>
       </c>
       <c r="G1" t="str">
-        <v>Image 1</v>
+        <v>Image 2</v>
       </c>
       <c r="H1" t="str">
-        <v>Image 2</v>
+        <v>Image 3</v>
       </c>
       <c r="I1" t="str">
-        <v>Image 3</v>
+        <v>Stock Status</v>
       </c>
       <c r="J1" t="str">
-        <v>Stock Status</v>
+        <v>Badge</v>
       </c>
       <c r="K1" t="str">
-        <v>Badge</v>
+        <v>Description</v>
       </c>
       <c r="L1" t="str">
-        <v>Description</v>
-      </c>
-      <c r="M1" t="str">
         <v>Featured</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>P-201</v>
+        <v>P201</v>
       </c>
       <c r="B2" t="str">
         <v>Hand painted Kerala Kasavu saree</v>
@@ -450,14 +447,14 @@
       <c r="C2" t="str">
         <v>Ladies Wear</v>
       </c>
-      <c r="D2" t="str">
-        <v>Kasavu Sarees</v>
+      <c r="D2">
+        <v>4200</v>
       </c>
       <c r="E2">
-        <v>4200</v>
-      </c>
-      <c r="F2">
         <v>4950</v>
+      </c>
+      <c r="F2" t="str">
+        <v>7_1788628563833-9707.png</v>
       </c>
       <c r="G2" t="str">
         <v>7_1788628563833-9707.png</v>
@@ -466,24 +463,21 @@
         <v>7_1788628563833-9707.png</v>
       </c>
       <c r="I2" t="str">
-        <v>7_1788628563833-9707.png</v>
+        <v>Made to Order</v>
       </c>
       <c r="J2" t="str">
-        <v>Made to Order</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="K2" t="str">
-        <v>Fresh Arrivals</v>
+        <v>NO RETURN</v>
       </c>
       <c r="L2" t="str">
-        <v>NO RETURN</v>
-      </c>
-      <c r="M2" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>NDS-MW-1001</v>
+        <v>P202</v>
       </c>
       <c r="B3" t="str">
         <v>Mens wear</v>
@@ -491,14 +485,14 @@
       <c r="C3" t="str">
         <v>Mens Wear</v>
       </c>
-      <c r="D3" t="str">
-        <v>Kasavu Mundu Sets</v>
+      <c r="D3">
+        <v>3000</v>
       </c>
       <c r="E3">
-        <v>3000</v>
-      </c>
-      <c r="F3">
         <v>0</v>
+      </c>
+      <c r="F3" t="str">
+        <v>8_1788531893736-8676.png</v>
       </c>
       <c r="G3" t="str">
         <v>8_1788531893736-8676.png</v>
@@ -507,24 +501,21 @@
         <v>8_1788531893736-8676.png</v>
       </c>
       <c r="I3" t="str">
-        <v>8_1788531893736-8676.png</v>
+        <v>In Stock</v>
       </c>
       <c r="J3" t="str">
-        <v>In Stock</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="K3" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Handcrafted designer creation by Naomika Design Studio.</v>
       </c>
       <c r="L3" t="str">
-        <v>Handcrafted designer creation by Naomika Design Studio.</v>
-      </c>
-      <c r="M3" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>NDS-CU-1001</v>
+        <v>P203</v>
       </c>
       <c r="B4" t="str">
         <v>Purple gown</v>
@@ -532,14 +523,14 @@
       <c r="C4" t="str">
         <v>Customization</v>
       </c>
-      <c r="D4" t="str">
-        <v>Bespoke Bridal Couture</v>
+      <c r="D4">
+        <v>17500</v>
       </c>
       <c r="E4">
-        <v>17500</v>
-      </c>
-      <c r="F4">
         <v>0</v>
+      </c>
+      <c r="F4" t="str">
+        <v>3_1788531630686-7753.jpeg</v>
       </c>
       <c r="G4" t="str">
         <v>3_1788531630686-7753.jpeg</v>
@@ -548,24 +539,21 @@
         <v>3_1788531630686-7753.jpeg</v>
       </c>
       <c r="I4" t="str">
-        <v>3_1788531630686-7753.jpeg</v>
+        <v>Limited Stock</v>
       </c>
       <c r="J4" t="str">
-        <v>Limited Stock</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="K4" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Handcrafted designer creation by Naomika Design Studio.</v>
       </c>
       <c r="L4" t="str">
-        <v>Handcrafted designer creation by Naomika Design Studio.</v>
-      </c>
-      <c r="M4" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>NDS-LW-1002</v>
+        <v>P204</v>
       </c>
       <c r="B5" t="str">
         <v>Ivory top and pant</v>
@@ -573,14 +561,14 @@
       <c r="C5" t="str">
         <v>Ladies Wear</v>
       </c>
-      <c r="D5" t="str">
-        <v>Co-Ord Sets</v>
+      <c r="D5">
+        <v>6500</v>
       </c>
       <c r="E5">
-        <v>6500</v>
-      </c>
-      <c r="F5">
         <v>0</v>
+      </c>
+      <c r="F5" t="str">
+        <v>1_1788531606882-8672.jpeg</v>
       </c>
       <c r="G5" t="str">
         <v>1_1788531606882-8672.jpeg</v>
@@ -589,24 +577,21 @@
         <v>1_1788531606882-8672.jpeg</v>
       </c>
       <c r="I5" t="str">
-        <v>1_1788531606882-8672.jpeg</v>
+        <v>In Stock</v>
       </c>
       <c r="J5" t="str">
-        <v>In Stock</v>
+        <v>Fresh Arrivals</v>
       </c>
       <c r="K5" t="str">
-        <v>Fresh Arrivals</v>
+        <v>Handcrafted designer creation by Naomika Design Studio.</v>
       </c>
       <c r="L5" t="str">
-        <v>Handcrafted designer creation by Naomika Design Studio.</v>
-      </c>
-      <c r="M5" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>NDS-LW-1001</v>
+        <v>P205</v>
       </c>
       <c r="B6" t="str">
         <v>MODAL SLIK KAFTAN</v>
@@ -614,14 +599,14 @@
       <c r="C6" t="str">
         <v>Customization</v>
       </c>
-      <c r="D6" t="str">
-        <v>Co-Ord Sets</v>
+      <c r="D6">
+        <v>7500</v>
       </c>
       <c r="E6">
-        <v>7500</v>
-      </c>
-      <c r="F6">
         <v>0</v>
+      </c>
+      <c r="F6" t="str">
+        <v>2_1788531469161-2419.jpeg</v>
       </c>
       <c r="G6" t="str">
         <v>2_1788531469161-2419.jpeg</v>
@@ -630,109 +615,24 @@
         <v>2_1788531469161-2419.jpeg</v>
       </c>
       <c r="I6" t="str">
-        <v>2_1788531469161-2419.jpeg</v>
+        <v>Made to Order</v>
       </c>
       <c r="J6" t="str">
-        <v>Made to Order</v>
-      </c>
-      <c r="K6" t="str">
         <v>Fresh Arrivals</v>
       </c>
-      <c r="L6" t="str" xml:space="preserve">
+      <c r="K6" t="str" xml:space="preserve">
         <v xml:space="preserve">Handcrafted designer creation by Naomika Design Studio.
 Neck hand worked
 above excel price will vary 500-1000 rs
 customization possible</v>
       </c>
-      <c r="M6" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>NDS-JW-1001</v>
-      </c>
-      <c r="B7" t="str">
-        <v>Royal Antique Temple Jewellery Choker Set</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Jewellery</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Bridal Chokers</v>
-      </c>
-      <c r="E7">
-        <v>18500</v>
-      </c>
-      <c r="F7">
-        <v>22000</v>
-      </c>
-      <c r="G7" t="str">
-        <v>kerala_bridal_jewellery.jpg</v>
-      </c>
-      <c r="H7" t="str">
-        <v>kerala_bridal_jewellery.jpg</v>
-      </c>
-      <c r="I7" t="str">
-        <v>kerala_bridal_jewellery.jpg</v>
-      </c>
-      <c r="J7" t="str">
-        <v>In Stock</v>
-      </c>
-      <c r="K7" t="str">
-        <v>Curated Release</v>
-      </c>
-      <c r="L7" t="str">
-        <v>Authentic 22K antique gold finish temple jewellery bridal choker necklace adorned with radiant ruby-red stones, emerald accents, south sea pearls, and matching handcrafted jhumkas.</v>
-      </c>
-      <c r="M7" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>NDS-JW-1002</v>
-      </c>
-      <c r="B8" t="str">
-        <v>Heritage Kasavu Coin Necklace &amp; Royal Bangles</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Jewellery</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Temple Jewellery</v>
-      </c>
-      <c r="E8">
-        <v>14200</v>
-      </c>
-      <c r="F8">
-        <v>16500</v>
-      </c>
-      <c r="G8" t="str">
-        <v>kerala_bridal_bangles.jpg</v>
-      </c>
-      <c r="H8" t="str">
-        <v>kerala_bridal_bangles.jpg</v>
-      </c>
-      <c r="I8" t="str">
-        <v>kerala_bridal_bangles.jpg</v>
-      </c>
-      <c r="J8" t="str">
-        <v>In Stock</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Curated Release</v>
-      </c>
-      <c r="L8" t="str">
-        <v>Traditional Kerala Palakka and Kasavu coin necklace paired with intricately sculpted antique temple kadas featuring Goddess Lakshmi motifs and gemstone inlays.</v>
-      </c>
-      <c r="M8" t="str">
+      <c r="L6" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:M8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add Size Selection in Admin Panel for LW/MW and enforce No Return Policy across all products
</commit_message>
<xml_diff>
--- a/products.xlsx
+++ b/products.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:M12"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -416,223 +416,495 @@
         <v>Original Price</v>
       </c>
       <c r="F1" t="str">
+        <v>Sizes</v>
+      </c>
+      <c r="G1" t="str">
         <v>Image 1</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>Image 2</v>
       </c>
-      <c r="H1" t="str">
+      <c r="I1" t="str">
         <v>Image 3</v>
       </c>
-      <c r="I1" t="str">
+      <c r="J1" t="str">
         <v>Stock Status</v>
       </c>
-      <c r="J1" t="str">
+      <c r="K1" t="str">
         <v>Badge</v>
       </c>
-      <c r="K1" t="str">
+      <c r="L1" t="str">
         <v>Description</v>
       </c>
-      <c r="L1" t="str">
+      <c r="M1" t="str">
         <v>Featured</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>P201</v>
+        <v>P211</v>
       </c>
       <c r="B2" t="str">
-        <v>Hand painted Kerala Kasavu saree</v>
+        <v>Crimson Gold Embellished Bridal Lehenga</v>
       </c>
       <c r="C2" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D2">
-        <v>4200</v>
+        <v>25000</v>
       </c>
       <c r="E2">
-        <v>4950</v>
+        <v>0</v>
       </c>
       <c r="F2" t="str">
-        <v>7_1788628563833-9707.png</v>
+        <v>S, M, L, XL</v>
       </c>
       <c r="G2" t="str">
-        <v>7_1788628563833-9707.png</v>
+        <v>10_1788721631854-5301.png</v>
       </c>
       <c r="H2" t="str">
-        <v>7_1788628563833-9707.png</v>
+        <v>10_1788721631854-5301.png</v>
       </c>
       <c r="I2" t="str">
-        <v>Made to Order</v>
+        <v>10_1788721631854-5301.png</v>
       </c>
       <c r="J2" t="str">
-        <v>Fresh Arrivals</v>
+        <v>In Stock</v>
       </c>
       <c r="K2" t="str">
-        <v>NO RETURN</v>
+        <v>Bridal Heritage</v>
       </c>
       <c r="L2" t="str">
+        <v>Exuding regal splendor, this opulent bridal ensemble features a richly detailed crimson blouse adorned with intricate zardozi hand embroidery and sheer embellished sleeves, paired with a shimmering woven gold lehenga skirt. Completed with a luxurious tissue dupatta, it is meticulously tailored for grand wedding receptions and evening celebrations. Note: No Return Policy.</v>
+      </c>
+      <c r="M2" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>P202</v>
+        <v>P210</v>
       </c>
       <c r="B3" t="str">
-        <v>Mens wear</v>
+        <v>Royal Blue Brocade Halter Blouse</v>
       </c>
       <c r="C3" t="str">
-        <v>Mens Wear</v>
+        <v>Ladies Wear</v>
       </c>
       <c r="D3">
-        <v>3000</v>
+        <v>4500</v>
       </c>
       <c r="E3">
         <v>0</v>
       </c>
       <c r="F3" t="str">
-        <v>8_1788531893736-8676.png</v>
+        <v>S, M, L, XL</v>
       </c>
       <c r="G3" t="str">
-        <v>8_1788531893736-8676.png</v>
+        <v>9_1788721582211-8463.png</v>
       </c>
       <c r="H3" t="str">
-        <v>8_1788531893736-8676.png</v>
+        <v>9_1788721582211-8463.png</v>
       </c>
       <c r="I3" t="str">
+        <v>9_1788721582211-8463.png</v>
+      </c>
+      <c r="J3" t="str">
         <v>In Stock</v>
       </c>
-      <c r="J3" t="str">
-        <v>Fresh Arrivals</v>
-      </c>
       <c r="K3" t="str">
-        <v>Handcrafted designer creation by Naomika Design Studio.</v>
+        <v>Festive Edit</v>
       </c>
       <c r="L3" t="str">
+        <v>Impeccably tailored from lustrous royal blue silk brocade, this high-neck halter blouse features intricate woven gold zari floral motifs that radiate contemporary charm. Perfectly paired with ivory kasavu drapes or festive lehengas, it offers a striking silhouette ideal for evening celebrations and wedding receptions. Note: No Return Policy.</v>
+      </c>
+      <c r="M3" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>P203</v>
+        <v>P209</v>
       </c>
       <c r="B4" t="str">
-        <v>Purple gown</v>
+        <v>Ivory Kasavu Striped Kurta Mundu Set</v>
       </c>
       <c r="C4" t="str">
-        <v>Customization</v>
+        <v>Mens Wear</v>
       </c>
       <c r="D4">
-        <v>17500</v>
+        <v>3500</v>
       </c>
       <c r="E4">
         <v>0</v>
       </c>
       <c r="F4" t="str">
-        <v>3_1788531630686-7753.jpeg</v>
+        <v/>
       </c>
       <c r="G4" t="str">
-        <v>3_1788531630686-7753.jpeg</v>
+        <v>8_1788721559495-2695.png</v>
       </c>
       <c r="H4" t="str">
-        <v>3_1788531630686-7753.jpeg</v>
+        <v>8_1788721559495-2695.png</v>
       </c>
       <c r="I4" t="str">
-        <v>Limited Stock</v>
+        <v>8_1788721559495-2695.png</v>
       </c>
       <c r="J4" t="str">
-        <v>Fresh Arrivals</v>
+        <v>In Stock</v>
       </c>
       <c r="K4" t="str">
-        <v>Handcrafted designer creation by Naomika Design Studio.</v>
+        <v>Festive Edit</v>
       </c>
       <c r="L4" t="str">
-        <v>Yes</v>
-      </c>
-    </row>
-    <row r="5">
+        <v>Imbued with understated elegance, this pristine off-white kurta features delicate vertical gold kasavu zari stripes for a refined festive charm. Paired impeccably with a traditional golden zari-bordered mundu, this ensemble honors Kerala's rich sartorial heritage with contemporary elegance. Perfect for Onam celebrations, traditional wedding ceremonies, and auspicious festive rituals.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="5" xml:space="preserve">
       <c r="A5" t="str">
-        <v>P204</v>
+        <v>P208</v>
       </c>
       <c r="B5" t="str">
-        <v>Ivory top and pant</v>
+        <v>Ivory Floral Hand-Painted Kasavu Saree</v>
       </c>
       <c r="C5" t="str">
         <v>Ladies Wear</v>
       </c>
       <c r="D5">
-        <v>6500</v>
+        <v>5000</v>
       </c>
       <c r="E5">
         <v>0</v>
       </c>
       <c r="F5" t="str">
-        <v>1_1788531606882-8672.jpeg</v>
+        <v>S, M, L, XL</v>
       </c>
       <c r="G5" t="str">
-        <v>1_1788531606882-8672.jpeg</v>
+        <v>7_1788721516950-7398.png</v>
       </c>
       <c r="H5" t="str">
-        <v>1_1788531606882-8672.jpeg</v>
+        <v>7_1788721516950-7398.png</v>
       </c>
       <c r="I5" t="str">
+        <v>7_1788721516950-7398.png</v>
+      </c>
+      <c r="J5" t="str">
         <v>In Stock</v>
       </c>
-      <c r="J5" t="str">
-        <v>Fresh Arrivals</v>
-      </c>
       <c r="K5" t="str">
-        <v>Handcrafted designer creation by Naomika Design Studio.</v>
-      </c>
-      <c r="L5" t="str">
+        <v>Handcrafted Couture</v>
+      </c>
+      <c r="L5" t="str" xml:space="preserve">
+        <v xml:space="preserve">This exquisite ivory Kasavu saree celebrates Kerala's rich heritage, beautifully adorned with delicate, hand-painted floral motifs in soft pink and leafy green hues. Crafted from premium handloom cotton, it features a classic golden zari border paired with a matching puff-sleeved blouse that exudes vintage grace. Perfect for Onam festivities, temple visits, or intimate wedding celebrations, this drape is a timeless ode to traditional elegance.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M5" t="str">
         <v>Yes</v>
       </c>
     </row>
     <row r="6" xml:space="preserve">
       <c r="A6" t="str">
-        <v>P205</v>
+        <v>P207</v>
       </c>
       <c r="B6" t="str">
-        <v>MODAL SLIK KAFTAN</v>
+        <v>Ivory Kasavu Embroidered Corset Gown</v>
       </c>
       <c r="C6" t="str">
         <v>Customization</v>
       </c>
       <c r="D6">
-        <v>7500</v>
+        <v>14000</v>
       </c>
       <c r="E6">
         <v>0</v>
       </c>
       <c r="F6" t="str">
+        <v>Custom Fit</v>
+      </c>
+      <c r="G6" t="str">
+        <v>5_1788721479116-3197.png</v>
+      </c>
+      <c r="H6" t="str">
+        <v>5_1788721479116-3197.png</v>
+      </c>
+      <c r="I6" t="str">
+        <v>5_1788721479116-3197.png</v>
+      </c>
+      <c r="J6" t="str">
+        <v>In Stock</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Bespoke Couture</v>
+      </c>
+      <c r="L6" t="str" xml:space="preserve">
+        <v xml:space="preserve">Reimagining traditional Kerala heritage with modern allure, this ivory gown features a structured strapless corset bodice delicately detailed with hand-embroidered golden motifs. Highlighted by classic golden Kasavu zari borders running down the fitted silhouette, it effortlessly blends regal grace with contemporary elegance. Perfectly suited for grand wedding receptions, engagement ceremonies, and opulent festive celebrations.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="7" xml:space="preserve">
+      <c r="A7" t="str">
+        <v>P206</v>
+      </c>
+      <c r="B7" t="str">
+        <v>Scarlet Embroidered Organza Fusion Set</v>
+      </c>
+      <c r="C7" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D7">
+        <v>3550</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7" t="str">
+        <v>S, M, L, XL</v>
+      </c>
+      <c r="G7" t="str">
+        <v>6_1788721385434-2405.png</v>
+      </c>
+      <c r="H7" t="str">
+        <v>6_1788721385434-2405.png</v>
+      </c>
+      <c r="I7" t="str">
+        <v>6_1788721385434-2405.png</v>
+      </c>
+      <c r="J7" t="str">
+        <v>In Stock</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Festive Edit</v>
+      </c>
+      <c r="L7" t="str" xml:space="preserve">
+        <v xml:space="preserve">Radiate contemporary elegance in this striking scarlet red fusion ensemble, featuring a tailored bustier paired with fluid trousers and a sheer organza longline jacket. The lightweight jacket is beautifully elevated by delicate scalloped gold zari embroidery tracing the borders and cuffs, adding a touch of traditional craftsmanship to a modern silhouette. Perfect for festive soirées, pre-wedding celebrations, or evening receptions, this ensemble effortlessly balances modern sophistication with timeless grace.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="8" xml:space="preserve">
+      <c r="A8" t="str">
+        <v>P201</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Hand painted Kerala Kasavu saree</v>
+      </c>
+      <c r="C8" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D8">
+        <v>4200</v>
+      </c>
+      <c r="E8">
+        <v>4950</v>
+      </c>
+      <c r="F8" t="str">
+        <v>S, M, L, XL</v>
+      </c>
+      <c r="G8" t="str">
+        <v>7_1788628563833-9707.png</v>
+      </c>
+      <c r="H8" t="str">
+        <v>7_1788628563833-9707.png</v>
+      </c>
+      <c r="I8" t="str">
+        <v>7_1788628563833-9707.png</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Made to Order</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Fresh Arrivals</v>
+      </c>
+      <c r="L8" t="str" xml:space="preserve">
+        <v xml:space="preserve">Handcrafted designer creation by Naomika Design Studio.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="9" xml:space="preserve">
+      <c r="A9" t="str">
+        <v>P202</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Mens wear</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Mens Wear</v>
+      </c>
+      <c r="D9">
+        <v>3000</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9" t="str">
+        <v>38 (S), 40 (M), 42 (L), 44 (XL)</v>
+      </c>
+      <c r="G9" t="str">
+        <v>8_1788531893736-8676.png</v>
+      </c>
+      <c r="H9" t="str">
+        <v>8_1788531893736-8676.png</v>
+      </c>
+      <c r="I9" t="str">
+        <v>8_1788531893736-8676.png</v>
+      </c>
+      <c r="J9" t="str">
+        <v>In Stock</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Fresh Arrivals</v>
+      </c>
+      <c r="L9" t="str" xml:space="preserve">
+        <v xml:space="preserve">Handcrafted designer creation by Naomika Design Studio.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="10" xml:space="preserve">
+      <c r="A10" t="str">
+        <v>P203</v>
+      </c>
+      <c r="B10" t="str">
+        <v>Purple gown</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Customization</v>
+      </c>
+      <c r="D10">
+        <v>17500</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Custom Fit</v>
+      </c>
+      <c r="G10" t="str">
+        <v>3_1788531630686-7753.jpeg</v>
+      </c>
+      <c r="H10" t="str">
+        <v>3_1788531630686-7753.jpeg</v>
+      </c>
+      <c r="I10" t="str">
+        <v>3_1788531630686-7753.jpeg</v>
+      </c>
+      <c r="J10" t="str">
+        <v>Limited Stock</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Fresh Arrivals</v>
+      </c>
+      <c r="L10" t="str" xml:space="preserve">
+        <v xml:space="preserve">Handcrafted designer creation by Naomika Design Studio.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M10" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="11" xml:space="preserve">
+      <c r="A11" t="str">
+        <v>P204</v>
+      </c>
+      <c r="B11" t="str">
+        <v>Ivory top and pant</v>
+      </c>
+      <c r="C11" t="str">
+        <v>Ladies Wear</v>
+      </c>
+      <c r="D11">
+        <v>6500</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11" t="str">
+        <v>S, M, L, XL</v>
+      </c>
+      <c r="G11" t="str">
+        <v>1_1788531606882-8672.jpeg</v>
+      </c>
+      <c r="H11" t="str">
+        <v>1_1788531606882-8672.jpeg</v>
+      </c>
+      <c r="I11" t="str">
+        <v>1_1788531606882-8672.jpeg</v>
+      </c>
+      <c r="J11" t="str">
+        <v>In Stock</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Fresh Arrivals</v>
+      </c>
+      <c r="L11" t="str" xml:space="preserve">
+        <v xml:space="preserve">Handcrafted designer creation by Naomika Design Studio.
+Note: No Return Policy.</v>
+      </c>
+      <c r="M11" t="str">
+        <v>Yes</v>
+      </c>
+    </row>
+    <row r="12" xml:space="preserve">
+      <c r="A12" t="str">
+        <v>P205</v>
+      </c>
+      <c r="B12" t="str">
+        <v>MODAL SLIK KAFTAN</v>
+      </c>
+      <c r="C12" t="str">
+        <v>Customization</v>
+      </c>
+      <c r="D12">
+        <v>7500</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Custom Fit</v>
+      </c>
+      <c r="G12" t="str">
         <v>2_1788531469161-2419.jpeg</v>
       </c>
-      <c r="G6" t="str">
+      <c r="H12" t="str">
         <v>2_1788531469161-2419.jpeg</v>
       </c>
-      <c r="H6" t="str">
+      <c r="I12" t="str">
         <v>2_1788531469161-2419.jpeg</v>
       </c>
-      <c r="I6" t="str">
+      <c r="J12" t="str">
         <v>Made to Order</v>
       </c>
-      <c r="J6" t="str">
+      <c r="K12" t="str">
         <v>Fresh Arrivals</v>
       </c>
-      <c r="K6" t="str" xml:space="preserve">
+      <c r="L12" t="str" xml:space="preserve">
         <v xml:space="preserve">Handcrafted designer creation by Naomika Design Studio.
 Neck hand worked
 above excel price will vary 500-1000 rs
-customization possible</v>
-      </c>
-      <c r="L6" t="str">
+customization possible
+Note: No Return Policy.</v>
+      </c>
+      <c r="M12" t="str">
         <v>Yes</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:L6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:M12"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>